<commit_message>
fix: supprime la contrainte note 0..1 ajoutée par Document Core bdd017bed550a65ba66048dc8af398f299ef354d
</commit_message>
<xml_diff>
--- a/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-allergy-intolerance.xlsx
+++ b/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-allergy-intolerance.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T09:28:38+00:00</t>
+    <t>2026-07-20T14:26:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -7406,7 +7406,7 @@
         <v>78</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
fix: backport AllergyIntolerance.type via extension xver R5→R4
FRCoreValueSetAllergyIntoleranceType contient des codes (idiosyncrasie,
hypersensibilité non allergique) interdits par le binding required de
AllergyIntolerance.type en R4. Ce binding passe à preferred en R5, donc
ces codes sont désormais portés via l'extension backport officielle
xver-r5.r4 (type.extension:type) plutôt que sur l'élément natif, qui
conserve son binding required R4 (allergy | intolerance).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> ed3e81c52c0f08ea286533bc40c96b2faceaf43c
</commit_message>
<xml_diff>
--- a/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-allergy-intolerance.xlsx
+++ b/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-allergy-intolerance.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2155" uniqueCount="431">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T15:52:32+00:00</t>
+    <t>2026-07-31T13:08:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -685,16 +685,99 @@
     <t>Allergic (typically immune-mediated) reactions have been traditionally regarded as an indicator for potential escalation to significant future risk. Contemporary knowledge suggests that some reactions previously thought to be immune-mediated are, in fact, non-immune, but in some cases can still pose a life threatening risk. It is acknowledged that many clinicians might not be in a position to distinguish the mechanism of a particular reaction. Often the term "allergy" is used rather generically and may overlap with the use of "intolerance" - in practice the boundaries between these two concepts might not be well-defined or understood. This data element is included nevertheless, because many legacy systems have captured this attribute. Immunologic testing may provide supporting evidence for the basis of the reaction and the causative substance, but no tests are 100% sensitive or specific for sensitivity to a particular substance. If, as is commonly the case, it is unclear whether the reaction is due to an allergy or an intolerance, then the type element should be omitted from the resource.</t>
   </si>
   <si>
+    <t>Identification of the underlying physiological mechanism for a Reaction Risk.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/allergy-intolerance-type|4.0.1</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>FiveWs.class</t>
+  </si>
+  <si>
+    <t>IAM-9</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>xml:id (or equivalent in JSON)</t>
+  </si>
+  <si>
+    <t>unique id for the element within a resource (for internal references)</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://hl7.org/fhir/5.0/StructureDefinition/extension-AllergyIntolerance.type|0.1.0}
+</t>
+  </si>
+  <si>
+    <t>Type d'allergie ou d'intolérance étendu (backport R5 : idiosyncrasie, hypersensibilité non allergique)</t>
+  </si>
+  <si>
+    <t>R5: `AllergyIntolerance.type` additional types (CodeableConcept) additional types from child elements (coding)</t>
+  </si>
+  <si>
+    <t>Element `AllergyIntolerance.type` is mapped to FHIR R4 element `AllergyIntolerance.type` as `SourceIsBroaderThanTarget`.
+The mappings for `AllergyIntolerance.type` do not cover the following types: CodeableConcept.
+The mappings for `AllergyIntolerance.type` do not cover the following types based on type expansion: coding.
+Allergic (typically immune-mediated) reactions have been traditionally regarded as an indicator for potential escalation to significant future risk. Contemporary knowledge suggests that some reactions previously thought to be immune-mediated are, in fact, non-immune, but in some cases can still pose a life threatening risk. It is acknowledged that many clinicians might not be in a position to distinguish the mechanism of a particular reaction. Often the term "allergy" is used rather generically and may overlap with the use of "intolerance" - in practice the boundaries between these two concepts might not be well-defined or understood. This data element is included nevertheless, because many legacy systems have captured this attribute. Immunologic testing may provide supporting evidence for the basis of the reaction and the causative substance, but no tests are 100% sensitive or specific for sensitivity to a particular substance. If, as is commonly the case, it is unclear whether the reaction is due to an allergy or an intolerance, then the type element should be omitted from the resource.</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.id</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.id</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.extension</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.extension</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.url</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.url</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/5.0/StructureDefinition/extension-AllergyIntolerance.type</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.value[x]</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.value[x]</t>
+  </si>
+  <si>
+    <t>allergy | intolerance - Underlying mechanism (if known)</t>
+  </si>
+  <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-allergy-intolerance-type|2.2.0</t>
   </si>
   <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>FiveWs.class</t>
-  </si>
-  <si>
-    <t>IAM-9</t>
+    <t>AllergyIntolerance.type.value</t>
+  </si>
+  <si>
+    <t>Primitive value for code</t>
+  </si>
+  <si>
+    <t>string.value</t>
   </si>
   <si>
     <t>AllergyIntolerance.category</t>
@@ -881,10 +964,6 @@
   </si>
   <si>
     <t>AllergyIntolerance.onset[x].id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">string
-</t>
   </si>
   <si>
     <t>AllergyIntolerance.onset[x]:onsetPeriod.extension</t>
@@ -1603,7 +1682,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AM53"/>
+  <dimension ref="A1:AM61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="52.0234375" customWidth="true" bestFit="true"/>
@@ -3820,9 +3899,11 @@
       <c r="X20" t="s" s="2">
         <v>197</v>
       </c>
-      <c r="Y20" s="2"/>
+      <c r="Y20" t="s" s="2">
+        <v>214</v>
+      </c>
       <c r="Z20" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>80</v>
@@ -3855,32 +3936,32 @@
         <v>100</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>219</v>
+        <v>80</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>80</v>
@@ -3889,20 +3970,18 @@
         <v>80</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>108</v>
+        <v>220</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="N21" t="s" s="2">
         <v>222</v>
       </c>
+      <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>80</v>
@@ -3927,13 +4006,13 @@
         <v>80</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>197</v>
+        <v>80</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>223</v>
+        <v>80</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>224</v>
+        <v>80</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>80</v>
@@ -3951,47 +4030,47 @@
         <v>80</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>218</v>
+        <v>150</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>225</v>
+        <v>80</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>216</v>
+        <v>80</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>226</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>228</v>
+        <v>80</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>80</v>
@@ -4000,20 +4079,18 @@
         <v>80</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>229</v>
+        <v>134</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>230</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>231</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>80</v>
@@ -4038,68 +4115,68 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>197</v>
+        <v>80</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>232</v>
+        <v>80</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>233</v>
+        <v>80</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="AC22" s="2"/>
       <c r="AD22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>227</v>
+        <v>156</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>234</v>
+        <v>80</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>235</v>
+        <v>80</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>236</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>237</v>
-      </c>
-      <c r="C23" s="2"/>
+        <v>223</v>
+      </c>
+      <c r="C23" t="s" s="2">
+        <v>225</v>
+      </c>
       <c r="D23" t="s" s="2">
-        <v>238</v>
+        <v>80</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>88</v>
@@ -4111,19 +4188,19 @@
         <v>80</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>193</v>
+        <v>226</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4149,11 +4226,13 @@
         <v>80</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>242</v>
-      </c>
-      <c r="Y23" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z23" t="s" s="2">
-        <v>243</v>
+        <v>80</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>80</v>
@@ -4171,44 +4250,44 @@
         <v>80</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>237</v>
+        <v>156</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI23" t="s" s="2">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>244</v>
+        <v>80</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>245</v>
+        <v>80</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>246</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>247</v>
+        <v>230</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>248</v>
+        <v>80</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>88</v>
@@ -4220,16 +4299,16 @@
         <v>80</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>249</v>
+        <v>220</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>250</v>
+        <v>148</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>251</v>
+        <v>149</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4280,10 +4359,10 @@
         <v>80</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>247</v>
+        <v>150</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>88</v>
@@ -4292,24 +4371,24 @@
         <v>80</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>252</v>
+        <v>152</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>253</v>
+        <v>80</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>254</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>255</v>
+        <v>232</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>255</v>
+        <v>233</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4320,7 +4399,7 @@
         <v>78</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>80</v>
@@ -4332,13 +4411,13 @@
         <v>80</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>256</v>
+        <v>133</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>257</v>
+        <v>134</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>258</v>
+        <v>135</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4377,37 +4456,37 @@
         <v>80</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>80</v>
+        <v>136</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>80</v>
+        <v>155</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>255</v>
+        <v>156</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>259</v>
+        <v>80</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>260</v>
+        <v>80</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>80</v>
@@ -4415,10 +4494,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>261</v>
+        <v>234</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>261</v>
+        <v>235</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4426,7 +4505,7 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G26" t="s" s="2">
         <v>88</v>
@@ -4441,22 +4520,24 @@
         <v>80</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>166</v>
+        <v>102</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>262</v>
+        <v>159</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="N26" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="N26" t="s" s="2">
+        <v>161</v>
+      </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q26" s="2"/>
       <c r="R26" t="s" s="2">
-        <v>80</v>
+        <v>236</v>
       </c>
       <c r="S26" t="s" s="2">
         <v>80</v>
@@ -4486,20 +4567,22 @@
         <v>80</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>169</v>
-      </c>
-      <c r="AC26" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="AD26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>264</v>
+        <v>80</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>261</v>
+        <v>163</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH26" t="s" s="2">
         <v>88</v>
@@ -4508,13 +4591,13 @@
         <v>80</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>265</v>
+        <v>131</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>266</v>
+        <v>80</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>80</v>
@@ -4522,14 +4605,12 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>267</v>
+        <v>237</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="C27" t="s" s="2">
-        <v>268</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
         <v>80</v>
       </c>
@@ -4550,15 +4631,17 @@
         <v>80</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>269</v>
+        <v>193</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>270</v>
+        <v>239</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="N27" s="2"/>
+        <v>212</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>213</v>
+      </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>80</v>
@@ -4583,13 +4666,11 @@
         <v>80</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="Y27" s="2"/>
       <c r="Z27" t="s" s="2">
-        <v>80</v>
+        <v>240</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>80</v>
@@ -4607,7 +4688,7 @@
         <v>80</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>261</v>
+        <v>170</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4622,10 +4703,10 @@
         <v>100</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>265</v>
+        <v>131</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>266</v>
+        <v>80</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>80</v>
@@ -4633,10 +4714,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>271</v>
+        <v>241</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>272</v>
+        <v>241</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4659,13 +4740,13 @@
         <v>80</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>273</v>
+        <v>220</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>148</v>
+        <v>242</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>149</v>
+        <v>242</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4716,7 +4797,7 @@
         <v>80</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>150</v>
+        <v>243</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4731,7 +4812,7 @@
         <v>80</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>152</v>
+        <v>80</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>80</v>
@@ -4742,14 +4823,14 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>274</v>
+        <v>244</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>275</v>
+        <v>244</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>177</v>
+        <v>245</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -4765,19 +4846,19 @@
         <v>80</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>276</v>
+        <v>246</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>277</v>
+        <v>247</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4803,31 +4884,31 @@
         <v>80</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>80</v>
+        <v>197</v>
       </c>
       <c r="Y29" t="s" s="2">
-        <v>80</v>
+        <v>249</v>
       </c>
       <c r="Z29" t="s" s="2">
-        <v>80</v>
+        <v>250</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB29" t="s" s="2">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="AC29" t="s" s="2">
-        <v>155</v>
+        <v>80</v>
       </c>
       <c r="AD29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE29" t="s" s="2">
-        <v>137</v>
+        <v>80</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>156</v>
+        <v>244</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -4839,32 +4920,32 @@
         <v>80</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>152</v>
+        <v>251</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>80</v>
+        <v>217</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>80</v>
+        <v>252</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>278</v>
+        <v>253</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>279</v>
+        <v>253</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>80</v>
+        <v>254</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G30" t="s" s="2">
         <v>88</v>
@@ -4879,16 +4960,16 @@
         <v>89</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>174</v>
+        <v>108</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>280</v>
+        <v>255</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>281</v>
+        <v>256</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>282</v>
+        <v>257</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4914,13 +4995,13 @@
         <v>80</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>80</v>
+        <v>197</v>
       </c>
       <c r="Y30" t="s" s="2">
-        <v>80</v>
+        <v>258</v>
       </c>
       <c r="Z30" t="s" s="2">
-        <v>80</v>
+        <v>259</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>80</v>
@@ -4938,7 +5019,7 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>283</v>
+        <v>253</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4947,35 +5028,35 @@
         <v>88</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>284</v>
+        <v>80</v>
       </c>
       <c r="AJ30" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>285</v>
+        <v>260</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>80</v>
+        <v>261</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>286</v>
+        <v>262</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>287</v>
+        <v>263</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>288</v>
+        <v>263</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>80</v>
+        <v>264</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>88</v>
@@ -4990,24 +5071,22 @@
         <v>89</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>289</v>
+        <v>265</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>290</v>
+        <v>266</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>291</v>
+        <v>267</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q31" t="s" s="2">
-        <v>292</v>
-      </c>
+      <c r="Q31" s="2"/>
       <c r="R31" t="s" s="2">
         <v>80</v>
       </c>
@@ -5027,13 +5106,11 @@
         <v>80</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y31" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>268</v>
+      </c>
+      <c r="Y31" s="2"/>
       <c r="Z31" t="s" s="2">
-        <v>80</v>
+        <v>269</v>
       </c>
       <c r="AA31" t="s" s="2">
         <v>80</v>
@@ -5051,7 +5128,7 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>293</v>
+        <v>263</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5060,37 +5137,35 @@
         <v>88</v>
       </c>
       <c r="AI31" t="s" s="2">
-        <v>284</v>
+        <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>294</v>
+        <v>270</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>80</v>
+        <v>271</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>295</v>
+        <v>272</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="C32" t="s" s="2">
-        <v>297</v>
-      </c>
+        <v>273</v>
+      </c>
+      <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G32" t="s" s="2">
         <v>88</v>
@@ -5102,16 +5177,16 @@
         <v>80</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>174</v>
+        <v>275</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5162,10 +5237,10 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="AG32" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH32" t="s" s="2">
         <v>88</v>
@@ -5177,21 +5252,21 @@
         <v>100</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>80</v>
+        <v>280</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5214,13 +5289,13 @@
         <v>80</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>174</v>
+        <v>282</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>300</v>
+        <v>283</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>301</v>
+        <v>284</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5271,7 +5346,7 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5286,25 +5361,25 @@
         <v>100</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>302</v>
+        <v>285</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>303</v>
+        <v>286</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>304</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>305</v>
+        <v>287</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>305</v>
+        <v>287</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>306</v>
+        <v>80</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5323,13 +5398,13 @@
         <v>80</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>307</v>
+        <v>166</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5368,19 +5443,17 @@
         <v>80</v>
       </c>
       <c r="AB34" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC34" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="AC34" s="2"/>
       <c r="AD34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>80</v>
+        <v>290</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>305</v>
+        <v>287</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5395,10 +5468,10 @@
         <v>100</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>310</v>
+        <v>291</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>311</v>
+        <v>292</v>
       </c>
       <c r="AM34" t="s" s="2">
         <v>80</v>
@@ -5406,14 +5479,16 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>312</v>
+        <v>293</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="C35" s="2"/>
+        <v>287</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>294</v>
+      </c>
       <c r="D35" t="s" s="2">
-        <v>313</v>
+        <v>80</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
@@ -5429,20 +5504,18 @@
         <v>80</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>314</v>
+        <v>295</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>315</v>
+        <v>296</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>316</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>317</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>80</v>
@@ -5491,7 +5564,7 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>312</v>
+        <v>287</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5506,21 +5579,21 @@
         <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>318</v>
+        <v>291</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>319</v>
+        <v>292</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>320</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>321</v>
+        <v>297</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>321</v>
+        <v>298</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5543,17 +5616,15 @@
         <v>80</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>174</v>
+        <v>220</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>322</v>
+        <v>148</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>324</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>80</v>
@@ -5602,7 +5673,7 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>321</v>
+        <v>150</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5614,10 +5685,10 @@
         <v>80</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>325</v>
+        <v>152</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>80</v>
@@ -5628,14 +5699,14 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>326</v>
+        <v>299</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>80</v>
+        <v>177</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5654,16 +5725,16 @@
         <v>80</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>327</v>
+        <v>133</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>328</v>
+        <v>301</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>329</v>
+        <v>302</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>330</v>
+        <v>180</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5701,19 +5772,19 @@
         <v>80</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>80</v>
+        <v>136</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>80</v>
+        <v>155</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>326</v>
+        <v>156</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5725,10 +5796,10 @@
         <v>80</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>331</v>
+        <v>152</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>80</v>
@@ -5739,10 +5810,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>332</v>
+        <v>303</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>332</v>
+        <v>304</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5750,7 +5821,7 @@
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G38" t="s" s="2">
         <v>88</v>
@@ -5762,18 +5833,20 @@
         <v>80</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>273</v>
+        <v>174</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>148</v>
+        <v>305</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>149</v>
-      </c>
-      <c r="N38" s="2"/>
+        <v>306</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>307</v>
+      </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>80</v>
@@ -5822,7 +5895,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>150</v>
+        <v>308</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5831,38 +5904,38 @@
         <v>88</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>80</v>
+        <v>309</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>152</v>
+        <v>310</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>80</v>
+        <v>311</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>333</v>
+        <v>312</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>177</v>
+        <v>80</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>80</v>
@@ -5871,25 +5944,27 @@
         <v>80</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>133</v>
+        <v>174</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>276</v>
+        <v>314</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>277</v>
+        <v>315</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>180</v>
+        <v>316</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q39" s="2"/>
+      <c r="Q39" t="s" s="2">
+        <v>317</v>
+      </c>
       <c r="R39" t="s" s="2">
         <v>80</v>
       </c>
@@ -5921,50 +5996,52 @@
         <v>80</v>
       </c>
       <c r="AB39" t="s" s="2">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="AC39" t="s" s="2">
-        <v>155</v>
+        <v>80</v>
       </c>
       <c r="AD39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE39" t="s" s="2">
-        <v>137</v>
+        <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>156</v>
+        <v>318</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>80</v>
+        <v>309</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>152</v>
+        <v>319</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>80</v>
+        <v>320</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>334</v>
+        <v>321</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="C40" s="2"/>
+        <v>287</v>
+      </c>
+      <c r="C40" t="s" s="2">
+        <v>322</v>
+      </c>
       <c r="D40" t="s" s="2">
         <v>80</v>
       </c>
@@ -5982,20 +6059,18 @@
         <v>80</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>335</v>
+        <v>174</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>336</v>
+        <v>323</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>338</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>80</v>
@@ -6044,7 +6119,7 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>339</v>
+        <v>287</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6059,21 +6134,21 @@
         <v>100</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>340</v>
+        <v>291</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>80</v>
+        <v>292</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>131</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>341</v>
+        <v>324</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>341</v>
+        <v>324</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6093,16 +6168,16 @@
         <v>80</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K41" t="s" s="2">
         <v>174</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>342</v>
+        <v>325</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>343</v>
+        <v>326</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6153,7 +6228,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>344</v>
+        <v>324</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6168,29 +6243,29 @@
         <v>100</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>345</v>
+        <v>327</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>80</v>
+        <v>328</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>131</v>
+        <v>329</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>80</v>
+        <v>331</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>88</v>
@@ -6202,16 +6277,16 @@
         <v>80</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>347</v>
+        <v>332</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>348</v>
+        <v>333</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>349</v>
+        <v>334</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6262,10 +6337,10 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH42" t="s" s="2">
         <v>88</v>
@@ -6277,32 +6352,32 @@
         <v>100</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>351</v>
+        <v>335</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>80</v>
+        <v>336</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>131</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>80</v>
+        <v>338</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>80</v>
@@ -6311,18 +6386,20 @@
         <v>80</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>353</v>
+        <v>339</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>354</v>
+        <v>340</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="N43" s="2"/>
+        <v>341</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>342</v>
+      </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>80</v>
@@ -6371,13 +6448,13 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>80</v>
@@ -6386,21 +6463,21 @@
         <v>100</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>356</v>
+        <v>343</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>80</v>
+        <v>344</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>80</v>
+        <v>345</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6423,15 +6500,17 @@
         <v>80</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>273</v>
+        <v>174</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>148</v>
+        <v>347</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>149</v>
-      </c>
-      <c r="N44" s="2"/>
+        <v>348</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>349</v>
+      </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>80</v>
@@ -6480,7 +6559,7 @@
         <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>150</v>
+        <v>346</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -6492,10 +6571,10 @@
         <v>80</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>152</v>
+        <v>350</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>80</v>
@@ -6506,14 +6585,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>177</v>
+        <v>80</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -6532,16 +6611,16 @@
         <v>80</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>133</v>
+        <v>352</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>276</v>
+        <v>353</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>277</v>
+        <v>354</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>180</v>
+        <v>355</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -6591,7 +6670,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>156</v>
+        <v>351</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6603,10 +6682,10 @@
         <v>80</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>152</v>
+        <v>356</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>80</v>
@@ -6617,46 +6696,42 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>360</v>
+        <v>80</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I46" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>133</v>
+        <v>220</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>361</v>
+        <v>148</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>362</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>181</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>80</v>
       </c>
@@ -6704,22 +6779,22 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>363</v>
+        <v>150</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>139</v>
+        <v>80</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>80</v>
@@ -6730,21 +6805,21 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
-        <v>80</v>
+        <v>177</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>80</v>
@@ -6756,16 +6831,16 @@
         <v>80</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>193</v>
+        <v>133</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>365</v>
+        <v>301</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>366</v>
+        <v>302</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>367</v>
+        <v>180</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6791,44 +6866,46 @@
         <v>80</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="Y47" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z47" t="s" s="2">
-        <v>368</v>
+        <v>80</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB47" t="s" s="2">
-        <v>80</v>
+        <v>136</v>
       </c>
       <c r="AC47" t="s" s="2">
-        <v>80</v>
+        <v>155</v>
       </c>
       <c r="AD47" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE47" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>364</v>
+        <v>156</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>369</v>
+        <v>152</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>80</v>
@@ -6839,21 +6916,21 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
-        <v>371</v>
+        <v>80</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>80</v>
@@ -6862,19 +6939,19 @@
         <v>80</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>193</v>
+        <v>360</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>373</v>
+        <v>362</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6900,13 +6977,13 @@
         <v>80</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>375</v>
+        <v>80</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>376</v>
+        <v>80</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>80</v>
@@ -6924,13 +7001,13 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>80</v>
@@ -6939,25 +7016,25 @@
         <v>100</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>215</v>
+        <v>365</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>377</v>
+        <v>131</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>379</v>
+        <v>80</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
@@ -6973,20 +7050,18 @@
         <v>80</v>
       </c>
       <c r="J49" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>273</v>
+        <v>174</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>380</v>
+        <v>367</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>381</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>382</v>
-      </c>
+        <v>368</v>
+      </c>
+      <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
         <v>80</v>
@@ -7035,7 +7110,7 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7050,21 +7125,21 @@
         <v>100</v>
       </c>
       <c r="AK49" t="s" s="2">
-        <v>383</v>
+        <v>370</v>
       </c>
       <c r="AL49" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>80</v>
+        <v>131</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7072,7 +7147,7 @@
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G50" t="s" s="2">
         <v>88</v>
@@ -7084,16 +7159,16 @@
         <v>80</v>
       </c>
       <c r="J50" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>174</v>
+        <v>372</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>386</v>
+        <v>374</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7144,10 +7219,10 @@
         <v>80</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="AG50" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH50" t="s" s="2">
         <v>88</v>
@@ -7159,21 +7234,21 @@
         <v>100</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>265</v>
+        <v>376</v>
       </c>
       <c r="AL50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM50" t="s" s="2">
-        <v>387</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7184,7 +7259,7 @@
         <v>78</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>80</v>
@@ -7196,17 +7271,15 @@
         <v>80</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>108</v>
+        <v>378</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>390</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>391</v>
-      </c>
+        <v>380</v>
+      </c>
+      <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
         <v>80</v>
@@ -7231,13 +7304,13 @@
         <v>80</v>
       </c>
       <c r="X51" t="s" s="2">
-        <v>197</v>
+        <v>80</v>
       </c>
       <c r="Y51" t="s" s="2">
-        <v>392</v>
+        <v>80</v>
       </c>
       <c r="Z51" t="s" s="2">
-        <v>393</v>
+        <v>80</v>
       </c>
       <c r="AA51" t="s" s="2">
         <v>80</v>
@@ -7255,13 +7328,13 @@
         <v>80</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>80</v>
@@ -7270,7 +7343,7 @@
         <v>100</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>234</v>
+        <v>381</v>
       </c>
       <c r="AL51" t="s" s="2">
         <v>80</v>
@@ -7281,10 +7354,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7307,17 +7380,15 @@
         <v>80</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>193</v>
+        <v>220</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>395</v>
+        <v>148</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>396</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>397</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
         <v>80</v>
@@ -7342,13 +7413,13 @@
         <v>80</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>398</v>
+        <v>80</v>
       </c>
       <c r="Y52" t="s" s="2">
-        <v>399</v>
+        <v>80</v>
       </c>
       <c r="Z52" t="s" s="2">
-        <v>400</v>
+        <v>80</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>80</v>
@@ -7366,7 +7437,7 @@
         <v>80</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>394</v>
+        <v>150</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>78</v>
@@ -7378,10 +7449,10 @@
         <v>80</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>401</v>
+        <v>152</v>
       </c>
       <c r="AL52" t="s" s="2">
         <v>80</v>
@@ -7392,14 +7463,14 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>402</v>
+        <v>383</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>402</v>
+        <v>383</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>80</v>
+        <v>177</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -7418,16 +7489,16 @@
         <v>80</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>327</v>
+        <v>133</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>403</v>
+        <v>301</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>404</v>
+        <v>302</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>405</v>
+        <v>180</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -7477,7 +7548,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>402</v>
+        <v>156</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7489,15 +7560,901 @@
         <v>80</v>
       </c>
       <c r="AJ53" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="AK53" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="AL53" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="B54" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" t="s" s="2">
+        <v>385</v>
+      </c>
+      <c r="E54" s="2"/>
+      <c r="F54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G54" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I54" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="J54" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="K54" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L54" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="M54" t="s" s="2">
+        <v>387</v>
+      </c>
+      <c r="N54" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="O54" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="P54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q54" s="2"/>
+      <c r="R54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF54" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="AG54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH54" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ54" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="AK54" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="AL54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="B55" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="C55" s="2"/>
+      <c r="D55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E55" s="2"/>
+      <c r="F55" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G55" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K55" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="L55" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="M55" t="s" s="2">
+        <v>391</v>
+      </c>
+      <c r="N55" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="O55" s="2"/>
+      <c r="P55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q55" s="2"/>
+      <c r="R55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X55" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="Y55" s="2"/>
+      <c r="Z55" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="AA55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF55" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="AG55" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH55" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ55" t="s" s="2">
         <v>100</v>
       </c>
-      <c r="AK53" t="s" s="2">
-        <v>331</v>
-      </c>
-      <c r="AL53" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM53" t="s" s="2">
+      <c r="AK55" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM55" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="2">
+        <v>395</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>395</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" t="s" s="2">
+        <v>396</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="G56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K56" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>397</v>
+      </c>
+      <c r="M56" t="s" s="2">
+        <v>398</v>
+      </c>
+      <c r="N56" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="O56" s="2"/>
+      <c r="P56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q56" s="2"/>
+      <c r="R56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X56" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="Y56" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="Z56" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="AA56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF56" t="s" s="2">
+        <v>395</v>
+      </c>
+      <c r="AG56" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AH56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ56" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK56" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="AL56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM56" t="s" s="2">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" t="s" s="2">
+        <v>404</v>
+      </c>
+      <c r="E57" s="2"/>
+      <c r="F57" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G57" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K57" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="L57" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="M57" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="N57" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="O57" s="2"/>
+      <c r="P57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q57" s="2"/>
+      <c r="R57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>408</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G58" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K58" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="L58" t="s" s="2">
+        <v>410</v>
+      </c>
+      <c r="M58" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="N58" s="2"/>
+      <c r="O58" s="2"/>
+      <c r="P58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q58" s="2"/>
+      <c r="R58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF58" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM58" t="s" s="2">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G59" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K59" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="N59" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="O59" s="2"/>
+      <c r="P59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q59" s="2"/>
+      <c r="R59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X59" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="Y59" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="Z59" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="AA59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF59" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AG59" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH59" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ59" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK59" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="AL59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM59" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G60" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K60" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="N60" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="O60" s="2"/>
+      <c r="P60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q60" s="2"/>
+      <c r="R60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X60" t="s" s="2">
+        <v>423</v>
+      </c>
+      <c r="Y60" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="Z60" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="AA60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF60" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="AG60" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH60" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ60" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK60" t="s" s="2">
+        <v>426</v>
+      </c>
+      <c r="AL60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM60" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="B61" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="D61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G61" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K61" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="L61" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="N61" t="s" s="2">
+        <v>430</v>
+      </c>
+      <c r="O61" s="2"/>
+      <c r="P61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q61" s="2"/>
+      <c r="R61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF61" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="AG61" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH61" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ61" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK61" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="AL61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM61" t="s" s="2">
         <v>80</v>
       </c>
     </row>

</xml_diff>